<commit_message>
feat: Customize Compressor numerical readings form and logs with the 6 user questions
</commit_message>
<xml_diff>
--- a/compressor_readings_log.xlsx
+++ b/compressor_readings_log.xlsx
@@ -1250,7 +1250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -1266,9 +1266,8 @@
       <c r="C1" s="23" t="n"/>
       <c r="D1" s="23" t="n"/>
       <c r="E1" s="23" t="n"/>
-      <c r="F1" s="23" t="n"/>
-      <c r="G1" s="24" t="n"/>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="F1" s="24" t="n"/>
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DOC NO: R/MAI/CR
 MONTH/YEAR: </t>
@@ -1286,8 +1285,7 @@
       <c r="D2" s="25" t="n"/>
       <c r="E2" s="25" t="n"/>
       <c r="F2" s="25" t="n"/>
-      <c r="G2" s="25" t="n"/>
-      <c r="H2" s="26" t="n"/>
+      <c r="G2" s="26" t="n"/>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -1297,7 +1295,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>RUN HOURS</t>
+          <t>RUNNING HOURS</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
@@ -1307,27 +1305,22 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>DISCHARGE PRESS</t>
+          <t>MOTOR HOURS</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>AIR TEMP</t>
+          <t>BAR</t>
         </is>
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>OIL TEMP</t>
+          <t>TEMPERATURE</t>
         </is>
       </c>
       <c r="G3" s="10" t="inlineStr">
         <is>
-          <t>MOTOR CURRENT</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
-        <is>
-          <t>OIL LEVEL</t>
+          <t>CARETAKER SIGN</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1334,6 @@
       <c r="E4" s="13" t="n"/>
       <c r="F4" s="13" t="n"/>
       <c r="G4" s="13" t="n"/>
-      <c r="H4" s="13" t="n"/>
     </row>
     <row r="5" ht="33" customHeight="1">
       <c r="A5" s="12" t="n">
@@ -1353,7 +1345,6 @@
       <c r="E5" s="13" t="n"/>
       <c r="F5" s="13" t="n"/>
       <c r="G5" s="13" t="n"/>
-      <c r="H5" s="13" t="n"/>
     </row>
     <row r="6" ht="33" customHeight="1">
       <c r="A6" s="12" t="n">
@@ -1365,7 +1356,6 @@
       <c r="E6" s="13" t="n"/>
       <c r="F6" s="13" t="n"/>
       <c r="G6" s="13" t="n"/>
-      <c r="H6" s="13" t="n"/>
     </row>
     <row r="7" ht="33" customHeight="1">
       <c r="A7" s="12" t="n">
@@ -1377,7 +1367,6 @@
       <c r="E7" s="13" t="n"/>
       <c r="F7" s="13" t="n"/>
       <c r="G7" s="13" t="n"/>
-      <c r="H7" s="13" t="n"/>
     </row>
     <row r="8" ht="33" customHeight="1">
       <c r="A8" s="12" t="n">
@@ -1389,7 +1378,6 @@
       <c r="E8" s="13" t="n"/>
       <c r="F8" s="13" t="n"/>
       <c r="G8" s="13" t="n"/>
-      <c r="H8" s="13" t="n"/>
     </row>
     <row r="9" ht="33" customHeight="1">
       <c r="A9" s="12" t="n">
@@ -1401,7 +1389,6 @@
       <c r="E9" s="13" t="n"/>
       <c r="F9" s="13" t="n"/>
       <c r="G9" s="13" t="n"/>
-      <c r="H9" s="13" t="n"/>
     </row>
     <row r="10" ht="33" customHeight="1">
       <c r="A10" s="15" t="n">
@@ -1413,7 +1400,6 @@
       <c r="E10" s="16" t="n"/>
       <c r="F10" s="16" t="n"/>
       <c r="G10" s="16" t="n"/>
-      <c r="H10" s="16" t="n"/>
     </row>
     <row r="11" ht="33" customHeight="1">
       <c r="A11" s="12" t="n">
@@ -1425,7 +1411,6 @@
       <c r="E11" s="13" t="n"/>
       <c r="F11" s="13" t="n"/>
       <c r="G11" s="13" t="n"/>
-      <c r="H11" s="13" t="n"/>
     </row>
     <row r="12" ht="33" customHeight="1">
       <c r="A12" s="12" t="n">
@@ -1437,7 +1422,6 @@
       <c r="E12" s="13" t="n"/>
       <c r="F12" s="13" t="n"/>
       <c r="G12" s="13" t="n"/>
-      <c r="H12" s="13" t="n"/>
     </row>
     <row r="13" ht="33" customHeight="1">
       <c r="A13" s="12" t="n">
@@ -1449,7 +1433,6 @@
       <c r="E13" s="13" t="n"/>
       <c r="F13" s="13" t="n"/>
       <c r="G13" s="13" t="n"/>
-      <c r="H13" s="13" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1">
       <c r="A14" s="12" t="n">
@@ -1461,7 +1444,6 @@
       <c r="E14" s="13" t="n"/>
       <c r="F14" s="13" t="n"/>
       <c r="G14" s="13" t="n"/>
-      <c r="H14" s="13" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1">
       <c r="A15" s="12" t="n">
@@ -1473,7 +1455,6 @@
       <c r="E15" s="13" t="n"/>
       <c r="F15" s="13" t="n"/>
       <c r="G15" s="13" t="n"/>
-      <c r="H15" s="13" t="n"/>
     </row>
     <row r="16" ht="33" customHeight="1">
       <c r="A16" s="12" t="n">
@@ -1485,7 +1466,6 @@
       <c r="E16" s="13" t="n"/>
       <c r="F16" s="13" t="n"/>
       <c r="G16" s="13" t="n"/>
-      <c r="H16" s="13" t="n"/>
     </row>
     <row r="17" ht="33" customHeight="1">
       <c r="A17" s="15" t="n">
@@ -1497,7 +1477,6 @@
       <c r="E17" s="16" t="n"/>
       <c r="F17" s="16" t="n"/>
       <c r="G17" s="16" t="n"/>
-      <c r="H17" s="16" t="n"/>
     </row>
     <row r="18" ht="33" customHeight="1">
       <c r="A18" s="12" t="n">
@@ -1509,7 +1488,6 @@
       <c r="E18" s="13" t="n"/>
       <c r="F18" s="13" t="n"/>
       <c r="G18" s="13" t="n"/>
-      <c r="H18" s="13" t="n"/>
     </row>
     <row r="19" ht="33" customHeight="1">
       <c r="A19" s="6" t="n"/>
@@ -1522,8 +1500,7 @@
       <c r="D19" s="25" t="n"/>
       <c r="E19" s="25" t="n"/>
       <c r="F19" s="25" t="n"/>
-      <c r="G19" s="25" t="n"/>
-      <c r="H19" s="26" t="n"/>
+      <c r="G19" s="26" t="n"/>
     </row>
     <row r="20" ht="59.25" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -1533,7 +1510,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>RUN HOURS</t>
+          <t>RUNNING HOURS</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -1543,27 +1520,22 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>DISCHARGE PRESS</t>
+          <t>MOTOR HOURS</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>AIR TEMP</t>
+          <t>BAR</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>OIL TEMP</t>
+          <t>TEMPERATURE</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>MOTOR CURRENT</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>OIL LEVEL</t>
+          <t>CARETAKER SIGN</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1549,6 @@
       <c r="E21" s="13" t="n"/>
       <c r="F21" s="13" t="n"/>
       <c r="G21" s="13" t="n"/>
-      <c r="H21" s="13" t="n"/>
     </row>
     <row r="22" ht="33" customHeight="1">
       <c r="A22" s="12" t="n">
@@ -1589,7 +1560,6 @@
       <c r="E22" s="13" t="n"/>
       <c r="F22" s="13" t="n"/>
       <c r="G22" s="13" t="n"/>
-      <c r="H22" s="13" t="n"/>
     </row>
     <row r="23" ht="33" customHeight="1">
       <c r="A23" s="12" t="n">
@@ -1601,7 +1571,6 @@
       <c r="E23" s="13" t="n"/>
       <c r="F23" s="13" t="n"/>
       <c r="G23" s="13" t="n"/>
-      <c r="H23" s="13" t="n"/>
     </row>
     <row r="24" ht="33" customHeight="1">
       <c r="A24" s="12" t="n">
@@ -1613,7 +1582,6 @@
       <c r="E24" s="13" t="n"/>
       <c r="F24" s="13" t="n"/>
       <c r="G24" s="13" t="n"/>
-      <c r="H24" s="13" t="n"/>
     </row>
     <row r="25" ht="33" customHeight="1">
       <c r="A25" s="12" t="n">
@@ -1625,7 +1593,6 @@
       <c r="E25" s="13" t="n"/>
       <c r="F25" s="13" t="n"/>
       <c r="G25" s="13" t="n"/>
-      <c r="H25" s="13" t="n"/>
     </row>
     <row r="26" ht="33" customHeight="1">
       <c r="A26" s="15" t="n">
@@ -1637,7 +1604,6 @@
       <c r="E26" s="16" t="n"/>
       <c r="F26" s="16" t="n"/>
       <c r="G26" s="16" t="n"/>
-      <c r="H26" s="16" t="n"/>
     </row>
     <row r="27" ht="33" customHeight="1">
       <c r="A27" s="12" t="n">
@@ -1649,7 +1615,6 @@
       <c r="E27" s="13" t="n"/>
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="13" t="n"/>
-      <c r="H27" s="13" t="n"/>
     </row>
     <row r="28" ht="33" customHeight="1">
       <c r="A28" s="12" t="n">
@@ -1661,7 +1626,6 @@
       <c r="E28" s="13" t="n"/>
       <c r="F28" s="13" t="n"/>
       <c r="G28" s="13" t="n"/>
-      <c r="H28" s="13" t="n"/>
     </row>
     <row r="29" ht="33" customHeight="1">
       <c r="A29" s="12" t="n">
@@ -1673,7 +1637,6 @@
       <c r="E29" s="13" t="n"/>
       <c r="F29" s="13" t="n"/>
       <c r="G29" s="13" t="n"/>
-      <c r="H29" s="13" t="n"/>
     </row>
     <row r="30" ht="33" customHeight="1">
       <c r="A30" s="12" t="n">
@@ -1685,7 +1648,6 @@
       <c r="E30" s="13" t="n"/>
       <c r="F30" s="13" t="n"/>
       <c r="G30" s="13" t="n"/>
-      <c r="H30" s="13" t="n"/>
     </row>
     <row r="31" ht="33" customHeight="1">
       <c r="A31" s="12" t="n">
@@ -1697,7 +1659,6 @@
       <c r="E31" s="13" t="n"/>
       <c r="F31" s="13" t="n"/>
       <c r="G31" s="13" t="n"/>
-      <c r="H31" s="13" t="n"/>
     </row>
     <row r="32" ht="33" customHeight="1">
       <c r="A32" s="12" t="n">
@@ -1709,7 +1670,6 @@
       <c r="E32" s="13" t="n"/>
       <c r="F32" s="13" t="n"/>
       <c r="G32" s="13" t="n"/>
-      <c r="H32" s="13" t="n"/>
     </row>
     <row r="33" ht="33" customHeight="1">
       <c r="A33" s="15" t="n">
@@ -1721,7 +1681,6 @@
       <c r="E33" s="16" t="n"/>
       <c r="F33" s="16" t="n"/>
       <c r="G33" s="16" t="n"/>
-      <c r="H33" s="16" t="n"/>
     </row>
     <row r="34" ht="33" customHeight="1">
       <c r="A34" s="12" t="n">
@@ -1733,7 +1692,6 @@
       <c r="E34" s="13" t="n"/>
       <c r="F34" s="13" t="n"/>
       <c r="G34" s="13" t="n"/>
-      <c r="H34" s="13" t="n"/>
     </row>
     <row r="35" ht="33" customHeight="1" thickBot="1">
       <c r="A35" s="12" t="n">
@@ -1745,7 +1703,6 @@
       <c r="E35" s="13" t="n"/>
       <c r="F35" s="13" t="n"/>
       <c r="G35" s="13" t="n"/>
-      <c r="H35" s="13" t="n"/>
     </row>
     <row r="36" ht="33" customHeight="1"/>
     <row r="37" ht="48.75" customHeight="1"/>
@@ -1763,10 +1720,10 @@
     <row r="55" ht="45" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="H1"/>
-    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>